<commit_message>
Switch enrichment to Anthropic-only, remove Gemini fallback
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/DB1_Creator_Profiles.xlsx
+++ b/data/DB1_Creator_Profiles.xlsx
@@ -813,17 +813,17 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>VC / Investor</t>
+          <t>Startup</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Venture Capital / Startups</t>
+          <t>Venture Capital</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -831,21 +831,17 @@
           <t>Established Creator</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>Global</t>
-        </is>
-      </c>
+      <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
         <v>0</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Contrarian</t>
+          <t>Tactical</t>
         </is>
       </c>
       <c r="O4" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q4" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update creator profiles and enriched data
</commit_message>
<xml_diff>
--- a/data/DB1_Creator_Profiles.xlsx
+++ b/data/DB1_Creator_Profiles.xlsx
@@ -735,12 +735,17 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-03-11</t>
+          <t>2026-03-28</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>FOUNDER</t>
+          <t>Startup</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>Global Health &amp; Clean Energy</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -748,8 +753,17 @@
           <t>Established Creator</t>
         </is>
       </c>
+      <c r="L3" t="inlineStr"/>
       <c r="M3" t="n">
         <v>0</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Data Driven</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="n">
+        <v>5</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
@@ -831,13 +845,12 @@
           <t>Established Creator</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr"/>
       <c r="M4" t="n">
         <v>0</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Tactical</t>
+          <t>Contrarian</t>
         </is>
       </c>
       <c r="O4" s="3" t="n">

</xml_diff>